<commit_message>
inclusión de sedimentos y data histórica de olas
</commit_message>
<xml_diff>
--- a/in/Sedimentos.xlsx
+++ b/in/Sedimentos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\Documents\dev\grafico_y_tablas_frecuencia\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCC40E5-5618-4F9A-BD4B-3779DFD163D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF351EE5-A3B8-421E-AC5C-6BA71D8EEF91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-9885" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot" sheetId="1" r:id="rId1"/>
@@ -221,7 +221,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -275,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -284,7 +284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -293,10 +293,12 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,12 +583,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="19.44140625" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" customWidth="1"/>
-    <col min="4" max="4" width="27.5546875" customWidth="1"/>
-    <col min="5" max="5" width="33.77734375" customWidth="1"/>
-    <col min="6" max="7" width="22.6640625" customWidth="1"/>
-    <col min="8" max="10" width="21.44140625" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" customWidth="1"/>
+    <col min="5" max="5" width="26.44140625" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" customWidth="1"/>
+    <col min="8" max="9" width="21.44140625" customWidth="1"/>
+    <col min="10" max="22" width="15.33203125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -889,43 +893,43 @@
       <c r="I5" s="2">
         <v>0.3</v>
       </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2">
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9">
         <v>2.85</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="9">
         <v>0.3</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="9">
         <v>11.33</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="9">
         <v>2.85</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5" s="9">
         <v>22.19</v>
       </c>
-      <c r="P5" s="2">
+      <c r="P5" s="9">
         <v>11.33</v>
       </c>
-      <c r="Q5" s="2">
+      <c r="Q5" s="9">
         <v>52.42</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="9">
         <v>22.19</v>
       </c>
-      <c r="S5" s="2">
+      <c r="S5" s="9">
         <v>10.47</v>
       </c>
-      <c r="T5" s="2">
+      <c r="T5" s="9">
         <v>52.42</v>
       </c>
-      <c r="U5" s="2">
+      <c r="U5" s="9">
         <v>0.65</v>
       </c>
-      <c r="V5" s="2">
+      <c r="V5" s="9">
         <v>10.47</v>
       </c>
     </row>
@@ -957,43 +961,43 @@
       <c r="I6" s="2">
         <v>0.38</v>
       </c>
-      <c r="J6" s="2">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2">
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9">
         <v>3.24</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="9">
         <v>0.38</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="9">
         <v>11.88</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="9">
         <v>3.24</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6" s="9">
         <v>20.96</v>
       </c>
-      <c r="P6" s="2">
+      <c r="P6" s="9">
         <v>11.88</v>
       </c>
-      <c r="Q6" s="2">
+      <c r="Q6" s="9">
         <v>52.12</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="9">
         <v>20.96</v>
       </c>
-      <c r="S6" s="2">
+      <c r="S6" s="9">
         <v>11.35</v>
       </c>
-      <c r="T6" s="2">
+      <c r="T6" s="9">
         <v>52.12</v>
       </c>
-      <c r="U6" s="2">
+      <c r="U6" s="9">
         <v>0.59</v>
       </c>
-      <c r="V6" s="2">
+      <c r="V6" s="9">
         <v>11.35</v>
       </c>
     </row>
@@ -1025,43 +1029,43 @@
       <c r="I7" s="2">
         <v>0.41</v>
       </c>
-      <c r="J7" s="2">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2">
+      <c r="J7" s="9">
+        <v>0</v>
+      </c>
+      <c r="K7" s="9">
         <v>1.38</v>
       </c>
-      <c r="L7" s="2">
+      <c r="L7" s="9">
         <v>0.41</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="9">
         <v>7.28</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="9">
         <v>1.38</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7" s="9">
         <v>18.190000000000001</v>
       </c>
-      <c r="P7" s="2">
+      <c r="P7" s="9">
         <v>7.28</v>
       </c>
-      <c r="Q7" s="2">
+      <c r="Q7" s="9">
         <v>57.78</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="9">
         <v>18.190000000000001</v>
       </c>
-      <c r="S7" s="2">
+      <c r="S7" s="9">
         <v>14.04</v>
       </c>
-      <c r="T7" s="2">
+      <c r="T7" s="9">
         <v>57.78</v>
       </c>
-      <c r="U7" s="2">
+      <c r="U7" s="9">
         <v>1.42</v>
       </c>
-      <c r="V7" s="2">
+      <c r="V7" s="9">
         <v>14.04</v>
       </c>
     </row>

</xml_diff>